<commit_message>
Add an order history
</commit_message>
<xml_diff>
--- a/assets/order_model.xlsx
+++ b/assets/order_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://abb-my.sharepoint.com/personal/baptiste_michot_be_abb_com/Documents/Documents/PrintersABB/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_66EEEB15BD16ADD4C2F9D051C49E0F7710D53F58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BD7D85D-74BA-441B-AF5E-995BD7675ADC}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_66EEEB15BD16ADD4C2F9D051C49E0F7710D53F58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC88389D-8EBD-4AA0-B942-BE25FDF21A95}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="297" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -104,18 +104,6 @@
     <t>EUR</t>
   </si>
   <si>
-    <t>HP 507X Toner Cartridge - Black - Laser - 11000 Page - 1 Each</t>
-  </si>
-  <si>
-    <t>HP 26X Toner Cartridge - Black - Laser - High Yield - 9000 Page - OEM</t>
-  </si>
-  <si>
-    <t>HP 59X - High Yield - black - original - LaserJet - toner cartridge</t>
-  </si>
-  <si>
-    <t>HP 149X High Yield Black Original LaserJet Toner Cartridge. Black toner page yield: 9500 pages, Printing colours: Black</t>
-  </si>
-  <si>
     <t>Invoice to:</t>
   </si>
   <si>
@@ -183,6 +171,9 @@
   </si>
   <si>
     <t>Advertising</t>
+  </si>
+  <si>
+    <t>Description</t>
   </si>
 </sst>
 </file>
@@ -647,105 +638,105 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -819,6 +810,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1200,9 +1195,9 @@
         <v>1</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="76"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="88"/>
     </row>
     <row r="4" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="49" t="s">
@@ -1215,79 +1210,79 @@
         <v>4</v>
       </c>
       <c r="I4" s="82"/>
-      <c r="J4" s="78"/>
+      <c r="J4" s="83"/>
     </row>
     <row r="5" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="49" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="51"/>
-      <c r="H5" s="73" t="s">
+      <c r="H5" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="70"/>
-      <c r="J5" s="65"/>
+      <c r="I5" s="85"/>
+      <c r="J5" s="86"/>
     </row>
     <row r="6" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="73" t="s">
+      <c r="H6" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="70"/>
-      <c r="J6" s="65"/>
+      <c r="I6" s="85"/>
+      <c r="J6" s="86"/>
     </row>
     <row r="7" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="73" t="s">
+      <c r="H7" s="84" t="s">
         <v>10</v>
       </c>
-      <c r="I7" s="70"/>
-      <c r="J7" s="65"/>
+      <c r="I7" s="85"/>
+      <c r="J7" s="86"/>
     </row>
     <row r="8" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="73"/>
-      <c r="I8" s="70"/>
-      <c r="J8" s="65"/>
+      <c r="H8" s="84"/>
+      <c r="I8" s="85"/>
+      <c r="J8" s="86"/>
     </row>
     <row r="9" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="73"/>
-      <c r="I9" s="70"/>
-      <c r="J9" s="65"/>
+      <c r="H9" s="84"/>
+      <c r="I9" s="85"/>
+      <c r="J9" s="86"/>
     </row>
     <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="49"/>
-      <c r="H10" s="73"/>
-      <c r="I10" s="70"/>
-      <c r="J10" s="65"/>
+      <c r="H10" s="84"/>
+      <c r="I10" s="85"/>
+      <c r="J10" s="86"/>
     </row>
     <row r="11" spans="1:10" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="49"/>
-      <c r="H11" s="73"/>
-      <c r="I11" s="70"/>
-      <c r="J11" s="65"/>
+      <c r="H11" s="84"/>
+      <c r="I11" s="85"/>
+      <c r="J11" s="86"/>
     </row>
     <row r="12" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="2"/>
-      <c r="C12" s="79" t="s">
+      <c r="C12" s="89" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="70"/>
-      <c r="H12" s="75"/>
-      <c r="I12" s="76"/>
-      <c r="J12" s="77"/>
+      <c r="D12" s="85"/>
+      <c r="H12" s="96"/>
+      <c r="I12" s="88"/>
+      <c r="J12" s="97"/>
     </row>
     <row r="13" spans="1:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
@@ -1301,11 +1296,11 @@
         <v>15</v>
       </c>
       <c r="B15" s="5"/>
-      <c r="C15" s="68">
+      <c r="C15" s="100">
         <f ca="1">TODAY()</f>
         <v>46104</v>
       </c>
-      <c r="D15" s="69"/>
+      <c r="D15" s="101"/>
     </row>
     <row r="16" spans="1:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I16" s="2"/>
@@ -1364,188 +1359,188 @@
       <c r="J21" s="14"/>
     </row>
     <row r="22" spans="1:13" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="88"/>
-      <c r="B22" s="89"/>
-      <c r="C22" s="89"/>
-      <c r="D22" s="89"/>
-      <c r="E22" s="90"/>
-      <c r="F22" s="90"/>
-      <c r="G22" s="90"/>
-      <c r="H22" s="88"/>
-      <c r="I22" s="91"/>
-      <c r="J22" s="92"/>
+      <c r="A22" s="66"/>
+      <c r="B22" s="67"/>
+      <c r="C22" s="67"/>
+      <c r="D22" s="67"/>
+      <c r="E22" s="68"/>
+      <c r="F22" s="68"/>
+      <c r="G22" s="68"/>
+      <c r="H22" s="66"/>
+      <c r="I22" s="98"/>
+      <c r="J22" s="99"/>
     </row>
     <row r="23" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="93">
+      <c r="A23" s="69">
         <v>1</v>
       </c>
-      <c r="B23" s="86" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="83"/>
-      <c r="D23" s="83"/>
-      <c r="E23" s="83"/>
-      <c r="F23" s="83"/>
-      <c r="G23" s="84"/>
-      <c r="H23" s="94">
+      <c r="B23" s="102" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="79"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="79"/>
+      <c r="F23" s="79"/>
+      <c r="G23" s="80"/>
+      <c r="H23" s="70">
         <v>238.3</v>
       </c>
-      <c r="I23" s="95">
+      <c r="I23" s="92">
         <f t="shared" ref="I23:I31" si="0">IF(H23="","",H23*A23)</f>
         <v>238.3</v>
       </c>
-      <c r="J23" s="84"/>
+      <c r="J23" s="80"/>
     </row>
     <row r="24" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="93">
+      <c r="A24" s="69">
         <v>1</v>
       </c>
-      <c r="B24" s="87" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="83"/>
-      <c r="D24" s="83"/>
-      <c r="E24" s="83"/>
-      <c r="F24" s="83"/>
-      <c r="G24" s="84"/>
-      <c r="H24" s="96">
+      <c r="B24" s="78" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="79"/>
+      <c r="D24" s="79"/>
+      <c r="E24" s="79"/>
+      <c r="F24" s="79"/>
+      <c r="G24" s="80"/>
+      <c r="H24" s="71">
         <v>234.65</v>
       </c>
-      <c r="I24" s="97">
+      <c r="I24" s="91">
         <f t="shared" si="0"/>
         <v>234.65</v>
       </c>
-      <c r="J24" s="84"/>
+      <c r="J24" s="80"/>
     </row>
     <row r="25" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="98">
+      <c r="A25" s="72">
         <v>4</v>
       </c>
-      <c r="B25" s="87" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="83"/>
-      <c r="D25" s="83"/>
-      <c r="E25" s="83"/>
-      <c r="F25" s="83"/>
-      <c r="G25" s="84"/>
-      <c r="H25" s="94">
+      <c r="B25" s="78" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="79"/>
+      <c r="D25" s="79"/>
+      <c r="E25" s="79"/>
+      <c r="F25" s="79"/>
+      <c r="G25" s="80"/>
+      <c r="H25" s="70">
         <v>233.9</v>
       </c>
-      <c r="I25" s="97">
+      <c r="I25" s="91">
         <f t="shared" si="0"/>
         <v>935.6</v>
       </c>
-      <c r="J25" s="84"/>
+      <c r="J25" s="80"/>
     </row>
     <row r="26" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="98">
+      <c r="A26" s="72">
         <v>1</v>
       </c>
-      <c r="B26" s="87" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" s="83"/>
-      <c r="D26" s="83"/>
-      <c r="E26" s="83"/>
-      <c r="F26" s="83"/>
-      <c r="G26" s="84"/>
-      <c r="H26" s="94">
+      <c r="B26" s="78" t="s">
+        <v>46</v>
+      </c>
+      <c r="C26" s="79"/>
+      <c r="D26" s="79"/>
+      <c r="E26" s="79"/>
+      <c r="F26" s="79"/>
+      <c r="G26" s="80"/>
+      <c r="H26" s="70">
         <v>217.37</v>
       </c>
-      <c r="I26" s="97">
+      <c r="I26" s="91">
         <f t="shared" si="0"/>
         <v>217.37</v>
       </c>
-      <c r="J26" s="84"/>
+      <c r="J26" s="80"/>
     </row>
     <row r="27" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="98"/>
-      <c r="B27" s="87"/>
-      <c r="C27" s="83"/>
-      <c r="D27" s="83"/>
-      <c r="E27" s="83"/>
-      <c r="F27" s="83"/>
-      <c r="G27" s="84"/>
-      <c r="H27" s="99"/>
-      <c r="I27" s="100" t="str">
+      <c r="A27" s="72"/>
+      <c r="B27" s="78"/>
+      <c r="C27" s="79"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="79"/>
+      <c r="F27" s="79"/>
+      <c r="G27" s="80"/>
+      <c r="H27" s="73"/>
+      <c r="I27" s="87" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J27" s="84"/>
+      <c r="J27" s="80"/>
     </row>
     <row r="28" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="98"/>
-      <c r="B28" s="87"/>
-      <c r="C28" s="83"/>
-      <c r="D28" s="83"/>
-      <c r="E28" s="83"/>
-      <c r="F28" s="83"/>
-      <c r="G28" s="84"/>
-      <c r="H28" s="101"/>
-      <c r="I28" s="100" t="str">
+      <c r="A28" s="72"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="79"/>
+      <c r="E28" s="79"/>
+      <c r="F28" s="79"/>
+      <c r="G28" s="80"/>
+      <c r="H28" s="74"/>
+      <c r="I28" s="87" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J28" s="84"/>
+      <c r="J28" s="80"/>
     </row>
     <row r="29" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="98"/>
-      <c r="B29" s="87"/>
-      <c r="C29" s="83"/>
-      <c r="D29" s="83"/>
-      <c r="E29" s="83"/>
-      <c r="F29" s="83"/>
-      <c r="G29" s="84"/>
-      <c r="H29" s="98"/>
-      <c r="I29" s="100" t="str">
+      <c r="A29" s="72"/>
+      <c r="B29" s="78"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="79"/>
+      <c r="E29" s="79"/>
+      <c r="F29" s="79"/>
+      <c r="G29" s="80"/>
+      <c r="H29" s="72"/>
+      <c r="I29" s="87" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J29" s="84"/>
+      <c r="J29" s="80"/>
       <c r="M29" s="63"/>
     </row>
     <row r="30" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="98"/>
-      <c r="B30" s="87"/>
-      <c r="C30" s="83"/>
-      <c r="D30" s="83"/>
-      <c r="E30" s="83"/>
-      <c r="F30" s="83"/>
-      <c r="G30" s="84"/>
-      <c r="H30" s="98"/>
-      <c r="I30" s="100" t="str">
+      <c r="A30" s="72"/>
+      <c r="B30" s="78"/>
+      <c r="C30" s="79"/>
+      <c r="D30" s="79"/>
+      <c r="E30" s="79"/>
+      <c r="F30" s="79"/>
+      <c r="G30" s="80"/>
+      <c r="H30" s="72"/>
+      <c r="I30" s="87" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J30" s="84"/>
+      <c r="J30" s="80"/>
     </row>
     <row r="31" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="98"/>
-      <c r="B31" s="87"/>
-      <c r="C31" s="83"/>
-      <c r="D31" s="83"/>
-      <c r="E31" s="83"/>
-      <c r="F31" s="83"/>
-      <c r="G31" s="84"/>
-      <c r="H31" s="98"/>
-      <c r="I31" s="100" t="str">
+      <c r="A31" s="72"/>
+      <c r="B31" s="78"/>
+      <c r="C31" s="79"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="79"/>
+      <c r="F31" s="79"/>
+      <c r="G31" s="80"/>
+      <c r="H31" s="72"/>
+      <c r="I31" s="87" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J31" s="84"/>
+      <c r="J31" s="80"/>
     </row>
     <row r="32" spans="1:13" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="102"/>
-      <c r="B32" s="85"/>
-      <c r="C32" s="85"/>
-      <c r="D32" s="85"/>
-      <c r="E32" s="85"/>
-      <c r="F32" s="85"/>
-      <c r="G32" s="85"/>
-      <c r="H32" s="102"/>
-      <c r="I32" s="103"/>
-      <c r="J32" s="104"/>
+      <c r="A32" s="75"/>
+      <c r="B32" s="65"/>
+      <c r="C32" s="65"/>
+      <c r="D32" s="65"/>
+      <c r="E32" s="65"/>
+      <c r="F32" s="65"/>
+      <c r="G32" s="65"/>
+      <c r="H32" s="75"/>
+      <c r="I32" s="93"/>
+      <c r="J32" s="94"/>
     </row>
     <row r="33" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="16"/>
@@ -1553,11 +1548,11 @@
       <c r="H33" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="I33" s="71">
+      <c r="I33" s="103">
         <f>SUM(I23:J32)</f>
         <v>1625.92</v>
       </c>
-      <c r="J33" s="65"/>
+      <c r="J33" s="86"/>
     </row>
     <row r="34" spans="1:10" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="17"/>
@@ -1573,16 +1568,16 @@
     </row>
     <row r="35" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="B35" s="80" t="s">
-        <v>28</v>
-      </c>
-      <c r="C35" s="67"/>
-      <c r="D35" s="67"/>
-      <c r="E35" s="65"/>
+        <v>23</v>
+      </c>
+      <c r="B35" s="95" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" s="77"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="86"/>
       <c r="F35" s="56" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G35" s="57"/>
       <c r="H35" s="57"/>
@@ -1592,7 +1587,7 @@
     <row r="36" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="24"/>
       <c r="F36" s="59" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G36" s="55"/>
       <c r="H36" s="60"/>
@@ -1601,31 +1596,31 @@
     </row>
     <row r="37" spans="1:10" s="3" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="66" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" s="67"/>
-      <c r="D37" s="67"/>
-      <c r="E37" s="67"/>
+        <v>27</v>
+      </c>
+      <c r="B37" s="90" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37" s="77"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
       <c r="F37" s="59" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G37" s="54"/>
-      <c r="H37" s="72"/>
-      <c r="I37" s="67"/>
+      <c r="H37" s="104"/>
+      <c r="I37" s="77"/>
       <c r="J37" s="44"/>
     </row>
     <row r="38" spans="1:10" s="3" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="24"/>
-      <c r="B38" s="74"/>
-      <c r="C38" s="67"/>
-      <c r="D38" s="67"/>
-      <c r="E38" s="67"/>
+      <c r="B38" s="76"/>
+      <c r="C38" s="77"/>
+      <c r="D38" s="77"/>
+      <c r="E38" s="77"/>
       <c r="F38" s="61"/>
       <c r="G38" s="52" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H38" s="53"/>
       <c r="I38" s="53"/>
@@ -1639,7 +1634,7 @@
       <c r="E39" s="45"/>
       <c r="F39" s="62"/>
       <c r="G39" s="52" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H39" s="53"/>
       <c r="I39" s="53"/>
@@ -1647,17 +1642,17 @@
     </row>
     <row r="40" spans="1:10" s="3" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="B40" s="66" t="s">
-        <v>37</v>
-      </c>
-      <c r="C40" s="67"/>
-      <c r="D40" s="67"/>
-      <c r="E40" s="67"/>
+        <v>32</v>
+      </c>
+      <c r="B40" s="90" t="s">
+        <v>33</v>
+      </c>
+      <c r="C40" s="77"/>
+      <c r="D40" s="77"/>
+      <c r="E40" s="77"/>
       <c r="F40" s="62"/>
       <c r="G40" s="52" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H40" s="53"/>
       <c r="I40" s="53"/>
@@ -1665,13 +1660,13 @@
     </row>
     <row r="41" spans="1:10" s="3" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="24"/>
-      <c r="B41" s="74"/>
-      <c r="C41" s="67"/>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
+      <c r="B41" s="76"/>
+      <c r="C41" s="77"/>
+      <c r="D41" s="77"/>
+      <c r="E41" s="77"/>
       <c r="F41" s="62"/>
       <c r="G41" s="52" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H41" s="53"/>
       <c r="I41" s="53"/>
@@ -1696,13 +1691,13 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B44" s="20"/>
       <c r="C44" s="20"/>
       <c r="D44" s="10"/>
       <c r="E44" s="9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F44" s="20"/>
       <c r="G44" s="18"/>
@@ -1718,7 +1713,7 @@
     </row>
     <row r="46" spans="1:10" s="32" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="31" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D46" s="33"/>
       <c r="E46" s="34"/>
@@ -1730,10 +1725,10 @@
       <c r="A47" s="31"/>
       <c r="D47" s="33"/>
       <c r="E47" s="34" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F47" s="32" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G47" s="33">
         <v>9981</v>
@@ -1743,14 +1738,14 @@
     </row>
     <row r="48" spans="1:10" s="32" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="31" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D48" s="33"/>
       <c r="E48" s="34" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F48" s="32" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G48" s="33">
         <v>9984</v>
@@ -1762,10 +1757,10 @@
       <c r="A49" s="31"/>
       <c r="D49" s="33"/>
       <c r="E49" s="34" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F49" s="32" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G49" s="32">
         <v>9977</v>
@@ -1777,10 +1772,10 @@
       <c r="A50" s="31"/>
       <c r="D50" s="33"/>
       <c r="E50" s="34" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F50" s="32" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G50" s="32">
         <v>9981</v>
@@ -1811,12 +1806,13 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="H37:I37"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="B30:G30"/>
     <mergeCell ref="B24:G24"/>
@@ -1833,6 +1829,12 @@
     <mergeCell ref="H10:J10"/>
     <mergeCell ref="B31:G31"/>
     <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="H6:J6"/>
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="I26:J26"/>
     <mergeCell ref="B29:G29"/>
@@ -1843,13 +1845,6 @@
     <mergeCell ref="H12:J12"/>
     <mergeCell ref="I22:J22"/>
     <mergeCell ref="I28:J28"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="H37:I37"/>
   </mergeCells>
   <pageMargins left="0.28000000000000003" right="0.27" top="0.31" bottom="0.3" header="0.17" footer="0.18"/>
   <pageSetup paperSize="9" scale="78" orientation="portrait"/>

</xml_diff>

<commit_message>
Add the possibility to send the order by mail
</commit_message>
<xml_diff>
--- a/assets/order_model.xlsx
+++ b/assets/order_model.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://abb-my.sharepoint.com/personal/baptiste_michot_be_abb_com/Documents/Documents/PrintersABB/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://abb-my.sharepoint.com/personal/baptiste_michot_be_abb_com/Documents/Documents/Imprimantes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_66EEEB15BD16ADD4C2F9D051C49E0F7710D53F58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC88389D-8EBD-4AA0-B942-BE25FDF21A95}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_66EEEB15BD16ADD4C2F9D051C49E0F7710D53F58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F7F50D3-C50A-46EE-86B4-2EE365C0859E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="297" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -671,60 +671,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -732,11 +686,57 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -809,11 +809,51 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>542572</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>16866</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>314417</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>63079</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B792049-B99F-C9C3-BD12-F98FD2DDEC0B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1864975" y="8413662"/>
+          <a:ext cx="1094248" cy="702791"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1195,9 +1235,9 @@
         <v>1</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="88"/>
-      <c r="I3" s="88"/>
-      <c r="J3" s="88"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
+      <c r="J3" s="87"/>
     </row>
     <row r="4" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="49" t="s">
@@ -1206,70 +1246,70 @@
       <c r="G4" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="81" t="s">
+      <c r="H4" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="82"/>
-      <c r="J4" s="83"/>
+      <c r="I4" s="99"/>
+      <c r="J4" s="100"/>
     </row>
     <row r="5" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="49" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="51"/>
-      <c r="H5" s="84" t="s">
+      <c r="H5" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="85"/>
-      <c r="J5" s="86"/>
+      <c r="I5" s="90"/>
+      <c r="J5" s="85"/>
     </row>
     <row r="6" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="84" t="s">
+      <c r="H6" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="85"/>
-      <c r="J6" s="86"/>
+      <c r="I6" s="90"/>
+      <c r="J6" s="85"/>
     </row>
     <row r="7" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="84" t="s">
+      <c r="H7" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="I7" s="85"/>
-      <c r="J7" s="86"/>
+      <c r="I7" s="90"/>
+      <c r="J7" s="85"/>
     </row>
     <row r="8" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="84"/>
-      <c r="I8" s="85"/>
-      <c r="J8" s="86"/>
+      <c r="H8" s="92"/>
+      <c r="I8" s="90"/>
+      <c r="J8" s="85"/>
     </row>
     <row r="9" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="84"/>
-      <c r="I9" s="85"/>
-      <c r="J9" s="86"/>
+      <c r="H9" s="92"/>
+      <c r="I9" s="90"/>
+      <c r="J9" s="85"/>
     </row>
     <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="49"/>
-      <c r="H10" s="84"/>
-      <c r="I10" s="85"/>
-      <c r="J10" s="86"/>
+      <c r="H10" s="92"/>
+      <c r="I10" s="90"/>
+      <c r="J10" s="85"/>
     </row>
     <row r="11" spans="1:10" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="49"/>
-      <c r="H11" s="84"/>
-      <c r="I11" s="85"/>
-      <c r="J11" s="86"/>
+      <c r="H11" s="92"/>
+      <c r="I11" s="90"/>
+      <c r="J11" s="85"/>
     </row>
     <row r="12" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
@@ -1279,10 +1319,10 @@
       <c r="C12" s="89" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="85"/>
-      <c r="H12" s="96"/>
-      <c r="I12" s="88"/>
-      <c r="J12" s="97"/>
+      <c r="D12" s="90"/>
+      <c r="H12" s="101"/>
+      <c r="I12" s="87"/>
+      <c r="J12" s="102"/>
     </row>
     <row r="13" spans="1:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
@@ -1296,11 +1336,11 @@
         <v>15</v>
       </c>
       <c r="B15" s="5"/>
-      <c r="C15" s="100">
+      <c r="C15" s="80">
         <f ca="1">TODAY()</f>
-        <v>46104</v>
-      </c>
-      <c r="D15" s="101"/>
+        <v>46105</v>
+      </c>
+      <c r="D15" s="81"/>
     </row>
     <row r="16" spans="1:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I16" s="2"/>
@@ -1367,42 +1407,42 @@
       <c r="F22" s="68"/>
       <c r="G22" s="68"/>
       <c r="H22" s="66"/>
-      <c r="I22" s="98"/>
-      <c r="J22" s="99"/>
+      <c r="I22" s="103"/>
+      <c r="J22" s="104"/>
     </row>
     <row r="23" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="69">
         <v>1</v>
       </c>
-      <c r="B23" s="102" t="s">
+      <c r="B23" s="82" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="79"/>
-      <c r="D23" s="79"/>
-      <c r="E23" s="79"/>
-      <c r="F23" s="79"/>
-      <c r="G23" s="80"/>
+      <c r="C23" s="83"/>
+      <c r="D23" s="83"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="77"/>
       <c r="H23" s="70">
         <v>238.3</v>
       </c>
-      <c r="I23" s="92">
+      <c r="I23" s="93">
         <f t="shared" ref="I23:I31" si="0">IF(H23="","",H23*A23)</f>
         <v>238.3</v>
       </c>
-      <c r="J23" s="80"/>
+      <c r="J23" s="77"/>
     </row>
     <row r="24" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="69">
         <v>1</v>
       </c>
-      <c r="B24" s="78" t="s">
+      <c r="B24" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="79"/>
-      <c r="D24" s="79"/>
-      <c r="E24" s="79"/>
-      <c r="F24" s="79"/>
-      <c r="G24" s="80"/>
+      <c r="C24" s="83"/>
+      <c r="D24" s="83"/>
+      <c r="E24" s="83"/>
+      <c r="F24" s="83"/>
+      <c r="G24" s="77"/>
       <c r="H24" s="71">
         <v>234.65</v>
       </c>
@@ -1410,20 +1450,20 @@
         <f t="shared" si="0"/>
         <v>234.65</v>
       </c>
-      <c r="J24" s="80"/>
+      <c r="J24" s="77"/>
     </row>
     <row r="25" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="72">
         <v>4</v>
       </c>
-      <c r="B25" s="78" t="s">
+      <c r="B25" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="C25" s="79"/>
-      <c r="D25" s="79"/>
-      <c r="E25" s="79"/>
-      <c r="F25" s="79"/>
-      <c r="G25" s="80"/>
+      <c r="C25" s="83"/>
+      <c r="D25" s="83"/>
+      <c r="E25" s="83"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="77"/>
       <c r="H25" s="70">
         <v>233.9</v>
       </c>
@@ -1431,20 +1471,20 @@
         <f t="shared" si="0"/>
         <v>935.6</v>
       </c>
-      <c r="J25" s="80"/>
+      <c r="J25" s="77"/>
     </row>
     <row r="26" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="72">
         <v>1</v>
       </c>
-      <c r="B26" s="78" t="s">
+      <c r="B26" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="79"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="79"/>
-      <c r="F26" s="79"/>
-      <c r="G26" s="80"/>
+      <c r="C26" s="83"/>
+      <c r="D26" s="83"/>
+      <c r="E26" s="83"/>
+      <c r="F26" s="83"/>
+      <c r="G26" s="77"/>
       <c r="H26" s="70">
         <v>217.37</v>
       </c>
@@ -1452,83 +1492,83 @@
         <f t="shared" si="0"/>
         <v>217.37</v>
       </c>
-      <c r="J26" s="80"/>
+      <c r="J26" s="77"/>
     </row>
     <row r="27" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="72"/>
-      <c r="B27" s="78"/>
-      <c r="C27" s="79"/>
-      <c r="D27" s="79"/>
-      <c r="E27" s="79"/>
-      <c r="F27" s="79"/>
-      <c r="G27" s="80"/>
+      <c r="B27" s="88"/>
+      <c r="C27" s="83"/>
+      <c r="D27" s="83"/>
+      <c r="E27" s="83"/>
+      <c r="F27" s="83"/>
+      <c r="G27" s="77"/>
       <c r="H27" s="73"/>
-      <c r="I27" s="87" t="str">
+      <c r="I27" s="76" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J27" s="80"/>
+      <c r="J27" s="77"/>
     </row>
     <row r="28" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="72"/>
-      <c r="B28" s="78"/>
-      <c r="C28" s="79"/>
-      <c r="D28" s="79"/>
-      <c r="E28" s="79"/>
-      <c r="F28" s="79"/>
-      <c r="G28" s="80"/>
+      <c r="B28" s="88"/>
+      <c r="C28" s="83"/>
+      <c r="D28" s="83"/>
+      <c r="E28" s="83"/>
+      <c r="F28" s="83"/>
+      <c r="G28" s="77"/>
       <c r="H28" s="74"/>
-      <c r="I28" s="87" t="str">
+      <c r="I28" s="76" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J28" s="80"/>
+      <c r="J28" s="77"/>
     </row>
     <row r="29" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="72"/>
-      <c r="B29" s="78"/>
-      <c r="C29" s="79"/>
-      <c r="D29" s="79"/>
-      <c r="E29" s="79"/>
-      <c r="F29" s="79"/>
-      <c r="G29" s="80"/>
+      <c r="B29" s="88"/>
+      <c r="C29" s="83"/>
+      <c r="D29" s="83"/>
+      <c r="E29" s="83"/>
+      <c r="F29" s="83"/>
+      <c r="G29" s="77"/>
       <c r="H29" s="72"/>
-      <c r="I29" s="87" t="str">
+      <c r="I29" s="76" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J29" s="80"/>
+      <c r="J29" s="77"/>
       <c r="M29" s="63"/>
     </row>
     <row r="30" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="72"/>
-      <c r="B30" s="78"/>
-      <c r="C30" s="79"/>
-      <c r="D30" s="79"/>
-      <c r="E30" s="79"/>
-      <c r="F30" s="79"/>
-      <c r="G30" s="80"/>
+      <c r="B30" s="88"/>
+      <c r="C30" s="83"/>
+      <c r="D30" s="83"/>
+      <c r="E30" s="83"/>
+      <c r="F30" s="83"/>
+      <c r="G30" s="77"/>
       <c r="H30" s="72"/>
-      <c r="I30" s="87" t="str">
+      <c r="I30" s="76" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J30" s="80"/>
+      <c r="J30" s="77"/>
     </row>
     <row r="31" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="72"/>
-      <c r="B31" s="78"/>
-      <c r="C31" s="79"/>
-      <c r="D31" s="79"/>
-      <c r="E31" s="79"/>
-      <c r="F31" s="79"/>
-      <c r="G31" s="80"/>
+      <c r="B31" s="88"/>
+      <c r="C31" s="83"/>
+      <c r="D31" s="83"/>
+      <c r="E31" s="83"/>
+      <c r="F31" s="83"/>
+      <c r="G31" s="77"/>
       <c r="H31" s="72"/>
-      <c r="I31" s="87" t="str">
+      <c r="I31" s="76" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J31" s="80"/>
+      <c r="J31" s="77"/>
     </row>
     <row r="32" spans="1:13" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="75"/>
@@ -1539,8 +1579,8 @@
       <c r="F32" s="65"/>
       <c r="G32" s="65"/>
       <c r="H32" s="75"/>
-      <c r="I32" s="93"/>
-      <c r="J32" s="94"/>
+      <c r="I32" s="94"/>
+      <c r="J32" s="95"/>
     </row>
     <row r="33" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="16"/>
@@ -1548,11 +1588,11 @@
       <c r="H33" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="I33" s="103">
+      <c r="I33" s="84">
         <f>SUM(I23:J32)</f>
         <v>1625.92</v>
       </c>
-      <c r="J33" s="86"/>
+      <c r="J33" s="85"/>
     </row>
     <row r="34" spans="1:10" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="17"/>
@@ -1570,12 +1610,12 @@
       <c r="A35" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="95" t="s">
+      <c r="B35" s="96" t="s">
         <v>24</v>
       </c>
-      <c r="C35" s="77"/>
-      <c r="D35" s="77"/>
-      <c r="E35" s="86"/>
+      <c r="C35" s="79"/>
+      <c r="D35" s="79"/>
+      <c r="E35" s="85"/>
       <c r="F35" s="56" t="s">
         <v>25</v>
       </c>
@@ -1598,26 +1638,26 @@
       <c r="A37" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B37" s="90" t="s">
+      <c r="B37" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="C37" s="77"/>
-      <c r="D37" s="77"/>
-      <c r="E37" s="77"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="79"/>
+      <c r="E37" s="79"/>
       <c r="F37" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G37" s="54"/>
-      <c r="H37" s="104"/>
-      <c r="I37" s="77"/>
+      <c r="H37" s="86"/>
+      <c r="I37" s="79"/>
       <c r="J37" s="44"/>
     </row>
     <row r="38" spans="1:10" s="3" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="24"/>
-      <c r="B38" s="76"/>
-      <c r="C38" s="77"/>
-      <c r="D38" s="77"/>
-      <c r="E38" s="77"/>
+      <c r="B38" s="97"/>
+      <c r="C38" s="79"/>
+      <c r="D38" s="79"/>
+      <c r="E38" s="79"/>
       <c r="F38" s="61"/>
       <c r="G38" s="52" t="s">
         <v>30</v>
@@ -1644,12 +1684,12 @@
       <c r="A40" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="B40" s="90" t="s">
+      <c r="B40" s="78" t="s">
         <v>33</v>
       </c>
-      <c r="C40" s="77"/>
-      <c r="D40" s="77"/>
-      <c r="E40" s="77"/>
+      <c r="C40" s="79"/>
+      <c r="D40" s="79"/>
+      <c r="E40" s="79"/>
       <c r="F40" s="62"/>
       <c r="G40" s="52" t="s">
         <v>34</v>
@@ -1660,10 +1700,10 @@
     </row>
     <row r="41" spans="1:10" s="3" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="24"/>
-      <c r="B41" s="76"/>
-      <c r="C41" s="77"/>
-      <c r="D41" s="77"/>
-      <c r="E41" s="77"/>
+      <c r="B41" s="97"/>
+      <c r="C41" s="79"/>
+      <c r="D41" s="79"/>
+      <c r="E41" s="79"/>
       <c r="F41" s="62"/>
       <c r="G41" s="52" t="s">
         <v>35</v>
@@ -1806,13 +1846,22 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I28:J28"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="B30:G30"/>
     <mergeCell ref="B24:G24"/>
@@ -1829,22 +1878,13 @@
     <mergeCell ref="H10:J10"/>
     <mergeCell ref="B31:G31"/>
     <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="H37:I37"/>
   </mergeCells>
   <pageMargins left="0.28000000000000003" right="0.27" top="0.31" bottom="0.3" header="0.17" footer="0.18"/>
   <pageSetup paperSize="9" scale="78" orientation="portrait"/>

</xml_diff>